<commit_message>
'fix: Restructure Notebooks and Update Results'
</commit_message>
<xml_diff>
--- a/Final Results Compiled/DB_Comparison.xlsx
+++ b/Final Results Compiled/DB_Comparison.xlsx
@@ -8,19 +8,33 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MS-MLAI-UpGrad\Research Things\LJMU Thesis\HotPotQA-Coding-Trials\Final Results Compiled\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93262683-FD8D-45CF-AA39-032543578C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{290F0833-418E-4405-93E5-E7F9EDA39D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiment Metrics" sheetId="1" r:id="rId1"/>
+    <sheet name="Ebedding Metrics" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="54">
   <si>
     <t>SN</t>
   </si>
@@ -124,15 +138,9 @@
     <t xml:space="preserve">  ▌ GraphRAG</t>
   </si>
   <si>
-    <t>GraphRAG</t>
-  </si>
-  <si>
     <t xml:space="preserve">  ▌ MultiStageGraphRAG</t>
   </si>
   <si>
-    <t>MultiStageGraphRAG</t>
-  </si>
-  <si>
     <t>Legend:</t>
   </si>
   <si>
@@ -149,6 +157,45 @@
   </si>
   <si>
     <t>RAGAS Faithfulness Rate</t>
+  </si>
+  <si>
+    <t>Multi-Stage Graph-Enhanced HybridRAG</t>
+  </si>
+  <si>
+    <t>Graph-Enhanced HybridRAG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ▌ VanillaRAG  (ChromaDB Fixed | Compared across Embedding Models)</t>
+  </si>
+  <si>
+    <t>No choice as no embedding is needed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ▌ SingleStageRAG  (ChromaDB Fixed | Compared across Embedding Models)</t>
+  </si>
+  <si>
+    <t>all-mpnet-base-v2</t>
+  </si>
+  <si>
+    <t>bge-base-en-v1.5</t>
+  </si>
+  <si>
+    <t>e5-base-v2</t>
+  </si>
+  <si>
+    <t>multi-qa-mpnet-base-cos-v1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ▌ MultiStageRAG  (ChromaDB Fixed | Compared across Embedding Models)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ▌ HybridRAG  (ChromaDB Fixed | Compared across Embedding Models)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ▌ GraphRAG  (ChromaDB Fixed | Compared across Embedding Models)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ▌ MultiStageGraphRAG  (ChromaDB Fixed | Compared across Embedding Models)</t>
   </si>
 </sst>
 </file>
@@ -158,7 +205,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -219,8 +266,44 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -293,8 +376,13 @@
         <fgColor theme="0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E75B6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -332,11 +420,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -391,10 +494,38 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -697,11 +828,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R35"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="3" width="22" customWidth="1"/>
+    <col min="2" max="2" width="39.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -766,7 +898,7 @@
         <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>15</v>
@@ -776,26 +908,26 @@
       </c>
     </row>
     <row r="2" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
     </row>
     <row r="3" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
@@ -814,7 +946,7 @@
         <v>20</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>22</v>
@@ -850,26 +982,26 @@
       <c r="R3" s="5"/>
     </row>
     <row r="4" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="21"/>
-      <c r="O4" s="21"/>
-      <c r="P4" s="21"/>
-      <c r="Q4" s="21"/>
-      <c r="R4" s="21"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="22"/>
     </row>
     <row r="5" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
@@ -1132,26 +1264,26 @@
       <c r="R9" s="3"/>
     </row>
     <row r="10" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="21"/>
-      <c r="N10" s="21"/>
-      <c r="O10" s="21"/>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="21"/>
-      <c r="R10" s="21"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="22"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
+      <c r="P10" s="22"/>
+      <c r="Q10" s="22"/>
+      <c r="R10" s="22"/>
     </row>
     <row r="11" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="13">
@@ -1414,26 +1546,26 @@
       <c r="R15" s="5"/>
     </row>
     <row r="16" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="21"/>
-      <c r="O16" s="21"/>
-      <c r="P16" s="21"/>
-      <c r="Q16" s="21"/>
-      <c r="R16" s="21"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="22"/>
+      <c r="P16" s="22"/>
+      <c r="Q16" s="22"/>
+      <c r="R16" s="22"/>
     </row>
     <row r="17" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
@@ -1696,33 +1828,33 @@
       <c r="R21" s="7"/>
     </row>
     <row r="22" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="21"/>
-      <c r="L22" s="21"/>
-      <c r="M22" s="21"/>
-      <c r="N22" s="21"/>
-      <c r="O22" s="21"/>
-      <c r="P22" s="21"/>
-      <c r="Q22" s="21"/>
-      <c r="R22" s="21"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="22"/>
+      <c r="J22" s="22"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="22"/>
+      <c r="N22" s="22"/>
+      <c r="O22" s="22"/>
+      <c r="P22" s="22"/>
+      <c r="Q22" s="22"/>
+      <c r="R22" s="22"/>
     </row>
     <row r="23" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16">
         <v>17</v>
       </c>
-      <c r="B23" s="5" t="s">
-        <v>34</v>
+      <c r="B23" s="20" t="s">
+        <v>42</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>19</v>
@@ -1773,8 +1905,8 @@
       <c r="A24" s="6">
         <v>18</v>
       </c>
-      <c r="B24" s="11" t="s">
-        <v>34</v>
+      <c r="B24" s="20" t="s">
+        <v>42</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>19</v>
@@ -1825,8 +1957,8 @@
       <c r="A25" s="16">
         <v>19</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>34</v>
+      <c r="B25" s="20" t="s">
+        <v>42</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>19</v>
@@ -1877,8 +2009,8 @@
       <c r="A26" s="10">
         <v>20</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>34</v>
+      <c r="B26" s="20" t="s">
+        <v>42</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>19</v>
@@ -1929,8 +2061,8 @@
       <c r="A27" s="16">
         <v>21</v>
       </c>
-      <c r="B27" s="3" t="s">
-        <v>34</v>
+      <c r="B27" s="20" t="s">
+        <v>42</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>19</v>
@@ -1978,33 +2110,33 @@
       <c r="R27" s="3"/>
     </row>
     <row r="28" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="B28" s="21"/>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
-      <c r="I28" s="21"/>
-      <c r="J28" s="21"/>
-      <c r="K28" s="21"/>
-      <c r="L28" s="21"/>
-      <c r="M28" s="21"/>
-      <c r="N28" s="21"/>
-      <c r="O28" s="21"/>
-      <c r="P28" s="21"/>
-      <c r="Q28" s="21"/>
-      <c r="R28" s="21"/>
+      <c r="A28" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="22"/>
+      <c r="J28" s="22"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="22"/>
+      <c r="M28" s="22"/>
+      <c r="N28" s="22"/>
+      <c r="O28" s="22"/>
+      <c r="P28" s="22"/>
+      <c r="Q28" s="22"/>
+      <c r="R28" s="22"/>
     </row>
     <row r="29" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>22</v>
       </c>
-      <c r="B29" s="7" t="s">
-        <v>36</v>
+      <c r="B29" s="20" t="s">
+        <v>41</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>19</v>
@@ -2055,8 +2187,8 @@
       <c r="A30" s="17">
         <v>23</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>36</v>
+      <c r="B30" s="20" t="s">
+        <v>41</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>19</v>
@@ -2107,8 +2239,8 @@
       <c r="A31" s="17">
         <v>24</v>
       </c>
-      <c r="B31" s="7" t="s">
-        <v>36</v>
+      <c r="B31" s="20" t="s">
+        <v>41</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>19</v>
@@ -2159,8 +2291,8 @@
       <c r="A32" s="10">
         <v>25</v>
       </c>
-      <c r="B32" s="11" t="s">
-        <v>36</v>
+      <c r="B32" s="20" t="s">
+        <v>41</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>19</v>
@@ -2211,8 +2343,8 @@
       <c r="A33" s="17">
         <v>26</v>
       </c>
-      <c r="B33" s="7" t="s">
-        <v>36</v>
+      <c r="B33" s="20" t="s">
+        <v>41</v>
       </c>
       <c r="C33" s="7" t="s">
         <v>19</v>
@@ -2261,16 +2393,60 @@
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A35" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C35" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="D35" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C35" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D35" s="19" t="s">
-        <v>40</v>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="L37" s="23">
+        <v>0.46350000000000002</v>
+      </c>
+      <c r="M37" s="8">
+        <v>0.45079999999999998</v>
+      </c>
+      <c r="N37">
+        <f>SUM(L37:M41)/10</f>
+        <v>0.47675999999999991</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="L38" s="24">
+        <v>0.47260000000000002</v>
+      </c>
+      <c r="M38" s="8">
+        <v>0.44030000000000002</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="L39" s="24">
+        <v>0.51859999999999995</v>
+      </c>
+      <c r="M39" s="12">
+        <v>0.4395</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="L40" s="25">
+        <v>0.56820000000000004</v>
+      </c>
+      <c r="M40" s="8">
+        <v>0.46310000000000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="L41" s="24">
+        <v>0.48749999999999999</v>
+      </c>
+      <c r="M41" s="4">
+        <v>0.46350000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -2284,4 +2460,1564 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9696554B-8C8E-4A6C-8CAC-D8E3C3A9927A}">
+  <dimension ref="A1:R37"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:18" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="26" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q1" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="26" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="3">
+        <v>100</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0.36</v>
+      </c>
+      <c r="I3" s="4">
+        <v>0.47539999999999999</v>
+      </c>
+      <c r="J3" s="4">
+        <v>0.15</v>
+      </c>
+      <c r="K3" s="4">
+        <v>0.51470000000000005</v>
+      </c>
+      <c r="L3" s="4">
+        <v>0.64329999999999998</v>
+      </c>
+      <c r="M3" s="4">
+        <v>0.45729999999999998</v>
+      </c>
+      <c r="N3" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="O3" s="4">
+        <v>0.31490000000000001</v>
+      </c>
+      <c r="P3" s="4">
+        <v>0.54300000000000004</v>
+      </c>
+      <c r="Q3" s="28"/>
+      <c r="R3" s="28" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A4" s="27" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="22"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A5" s="29">
+        <v>6</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="29">
+        <v>100</v>
+      </c>
+      <c r="E5" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="23">
+        <v>0.36</v>
+      </c>
+      <c r="I5" s="23">
+        <v>0.46350000000000002</v>
+      </c>
+      <c r="J5" s="23">
+        <v>0.11</v>
+      </c>
+      <c r="K5" s="23">
+        <v>0.46429999999999999</v>
+      </c>
+      <c r="L5" s="23">
+        <v>0.58830000000000005</v>
+      </c>
+      <c r="M5" s="23">
+        <v>0.40649999999999997</v>
+      </c>
+      <c r="N5" s="23">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="O5" s="23">
+        <v>0.30020000000000002</v>
+      </c>
+      <c r="P5" s="23">
+        <v>0.59419999999999995</v>
+      </c>
+      <c r="Q5" s="29"/>
+      <c r="R5" s="29"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A6" s="30">
+        <v>7</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="30">
+        <v>100</v>
+      </c>
+      <c r="E6" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="24">
+        <v>0.33</v>
+      </c>
+      <c r="I6" s="24">
+        <v>0.47260000000000002</v>
+      </c>
+      <c r="J6" s="24">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="K6" s="24">
+        <v>0.51580000000000004</v>
+      </c>
+      <c r="L6" s="24">
+        <v>0.67500000000000004</v>
+      </c>
+      <c r="M6" s="24">
+        <v>0.44400000000000001</v>
+      </c>
+      <c r="N6" s="24">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="O6" s="24">
+        <v>0.32019999999999998</v>
+      </c>
+      <c r="P6" s="24">
+        <v>0.64170000000000005</v>
+      </c>
+      <c r="Q6" s="30"/>
+      <c r="R6" s="30"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A7" s="30">
+        <v>8</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="30">
+        <v>100</v>
+      </c>
+      <c r="E7" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="24">
+        <v>0.37</v>
+      </c>
+      <c r="I7" s="24">
+        <v>0.51859999999999995</v>
+      </c>
+      <c r="J7" s="24">
+        <v>0.22</v>
+      </c>
+      <c r="K7" s="24">
+        <v>0.61409999999999998</v>
+      </c>
+      <c r="L7" s="24">
+        <v>0.73170000000000002</v>
+      </c>
+      <c r="M7" s="24">
+        <v>0.56030000000000002</v>
+      </c>
+      <c r="N7" s="24">
+        <v>0.13</v>
+      </c>
+      <c r="O7" s="24">
+        <v>0.38979999999999998</v>
+      </c>
+      <c r="P7" s="24">
+        <v>0.70309999999999995</v>
+      </c>
+      <c r="Q7" s="30"/>
+      <c r="R7" s="30"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A8" s="31">
+        <v>9</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="31">
+        <v>100</v>
+      </c>
+      <c r="E8" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" s="25">
+        <v>0.42</v>
+      </c>
+      <c r="I8" s="25">
+        <v>0.56820000000000004</v>
+      </c>
+      <c r="J8" s="25">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="K8" s="25">
+        <v>0.63009999999999999</v>
+      </c>
+      <c r="L8" s="25">
+        <v>0.745</v>
+      </c>
+      <c r="M8" s="25">
+        <v>0.57450000000000001</v>
+      </c>
+      <c r="N8" s="25">
+        <v>0.19</v>
+      </c>
+      <c r="O8" s="25">
+        <v>0.44729999999999998</v>
+      </c>
+      <c r="P8" s="25">
+        <v>0.71330000000000005</v>
+      </c>
+      <c r="Q8" s="31"/>
+      <c r="R8" s="31"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A9" s="30">
+        <v>10</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="30">
+        <v>100</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" s="24">
+        <v>0.36</v>
+      </c>
+      <c r="I9" s="24">
+        <v>0.48749999999999999</v>
+      </c>
+      <c r="J9" s="24">
+        <v>0.16</v>
+      </c>
+      <c r="K9" s="24">
+        <v>0.51929999999999998</v>
+      </c>
+      <c r="L9" s="24">
+        <v>0.66749999999999998</v>
+      </c>
+      <c r="M9" s="24">
+        <v>0.45569999999999999</v>
+      </c>
+      <c r="N9" s="24">
+        <v>0.1</v>
+      </c>
+      <c r="O9" s="24">
+        <v>0.33019999999999999</v>
+      </c>
+      <c r="P9" s="24">
+        <v>0.61329999999999996</v>
+      </c>
+      <c r="Q9" s="30"/>
+      <c r="R9" s="30"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A11" s="27" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
+      <c r="I11" s="22"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="22"/>
+      <c r="L11" s="22"/>
+      <c r="M11" s="22"/>
+      <c r="N11" s="22"/>
+      <c r="O11" s="22"/>
+      <c r="P11" s="22"/>
+      <c r="Q11" s="22"/>
+      <c r="R11" s="22"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A12" s="29">
+        <v>11</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="29">
+        <v>100</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" s="23">
+        <v>0.35</v>
+      </c>
+      <c r="I12" s="23">
+        <v>0.4894</v>
+      </c>
+      <c r="J12" s="23">
+        <v>0.21</v>
+      </c>
+      <c r="K12" s="23">
+        <v>0.54310000000000003</v>
+      </c>
+      <c r="L12" s="23">
+        <v>0.64080000000000004</v>
+      </c>
+      <c r="M12" s="23">
+        <v>0.50570000000000004</v>
+      </c>
+      <c r="N12" s="23">
+        <v>0.13</v>
+      </c>
+      <c r="O12" s="23">
+        <v>0.34599999999999997</v>
+      </c>
+      <c r="P12" s="23">
+        <v>0.65069999999999995</v>
+      </c>
+      <c r="Q12" s="29"/>
+      <c r="R12" s="29"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A13" s="30">
+        <v>12</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="30">
+        <v>100</v>
+      </c>
+      <c r="E13" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H13" s="24">
+        <v>0.44</v>
+      </c>
+      <c r="I13" s="24">
+        <v>0.58730000000000004</v>
+      </c>
+      <c r="J13" s="24">
+        <v>0.22</v>
+      </c>
+      <c r="K13" s="24">
+        <v>0.5786</v>
+      </c>
+      <c r="L13" s="24">
+        <v>0.7117</v>
+      </c>
+      <c r="M13" s="24">
+        <v>0.51729999999999998</v>
+      </c>
+      <c r="N13" s="24">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="O13" s="24">
+        <v>0.41899999999999998</v>
+      </c>
+      <c r="P13" s="24">
+        <v>0.6492</v>
+      </c>
+      <c r="Q13" s="30"/>
+      <c r="R13" s="30"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A14" s="30">
+        <v>13</v>
+      </c>
+      <c r="B14" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" s="30">
+        <v>100</v>
+      </c>
+      <c r="E14" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H14" s="24">
+        <v>0.45</v>
+      </c>
+      <c r="I14" s="24">
+        <v>0.58660000000000001</v>
+      </c>
+      <c r="J14" s="24">
+        <v>0.32</v>
+      </c>
+      <c r="K14" s="24">
+        <v>0.64180000000000004</v>
+      </c>
+      <c r="L14" s="24">
+        <v>0.72250000000000003</v>
+      </c>
+      <c r="M14" s="24">
+        <v>0.60229999999999995</v>
+      </c>
+      <c r="N14" s="24">
+        <v>0.17</v>
+      </c>
+      <c r="O14" s="24">
+        <v>0.4476</v>
+      </c>
+      <c r="P14" s="24">
+        <v>0.77110000000000001</v>
+      </c>
+      <c r="Q14" s="30"/>
+      <c r="R14" s="30"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A15" s="31">
+        <v>14</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="31">
+        <v>100</v>
+      </c>
+      <c r="E15" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H15" s="25">
+        <v>0.45</v>
+      </c>
+      <c r="I15" s="25">
+        <v>0.60970000000000002</v>
+      </c>
+      <c r="J15" s="25">
+        <v>0.31</v>
+      </c>
+      <c r="K15" s="25">
+        <v>0.62890000000000001</v>
+      </c>
+      <c r="L15" s="25">
+        <v>0.72170000000000001</v>
+      </c>
+      <c r="M15" s="25">
+        <v>0.58479999999999999</v>
+      </c>
+      <c r="N15" s="25">
+        <v>0.19</v>
+      </c>
+      <c r="O15" s="25">
+        <v>0.45910000000000001</v>
+      </c>
+      <c r="P15" s="25">
+        <v>0.70399999999999996</v>
+      </c>
+      <c r="Q15" s="31"/>
+      <c r="R15" s="31"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A16" s="30">
+        <v>15</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="30">
+        <v>100</v>
+      </c>
+      <c r="E16" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H16" s="24">
+        <v>0.38</v>
+      </c>
+      <c r="I16" s="24">
+        <v>0.53320000000000001</v>
+      </c>
+      <c r="J16" s="24">
+        <v>0.21</v>
+      </c>
+      <c r="K16" s="24">
+        <v>0.56089999999999995</v>
+      </c>
+      <c r="L16" s="24">
+        <v>0.66830000000000001</v>
+      </c>
+      <c r="M16" s="24">
+        <v>0.51149999999999995</v>
+      </c>
+      <c r="N16" s="24">
+        <v>0.11</v>
+      </c>
+      <c r="O16" s="24">
+        <v>0.373</v>
+      </c>
+      <c r="P16" s="24">
+        <v>0.60750000000000004</v>
+      </c>
+      <c r="Q16" s="30"/>
+      <c r="R16" s="30"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A18" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
+      <c r="L18" s="22"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="22"/>
+      <c r="P18" s="22"/>
+      <c r="Q18" s="22"/>
+      <c r="R18" s="22"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A19" s="30">
+        <v>16</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" s="30">
+        <v>100</v>
+      </c>
+      <c r="E19" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H19" s="24">
+        <v>0.41</v>
+      </c>
+      <c r="I19" s="24">
+        <v>0.51300000000000001</v>
+      </c>
+      <c r="J19" s="24">
+        <v>0.18</v>
+      </c>
+      <c r="K19" s="24">
+        <v>0.56659999999999999</v>
+      </c>
+      <c r="L19" s="24">
+        <v>0.6875</v>
+      </c>
+      <c r="M19" s="24">
+        <v>0.51819999999999999</v>
+      </c>
+      <c r="N19" s="24">
+        <v>0.12</v>
+      </c>
+      <c r="O19" s="24">
+        <v>0.35859999999999997</v>
+      </c>
+      <c r="P19" s="24">
+        <v>0.61919999999999997</v>
+      </c>
+      <c r="Q19" s="30"/>
+      <c r="R19" s="30"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A20" s="29">
+        <v>17</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="29">
+        <v>100</v>
+      </c>
+      <c r="E20" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="H20" s="23">
+        <v>0.38</v>
+      </c>
+      <c r="I20" s="23">
+        <v>0.51139999999999997</v>
+      </c>
+      <c r="J20" s="23">
+        <v>0.21</v>
+      </c>
+      <c r="K20" s="23">
+        <v>0.56640000000000001</v>
+      </c>
+      <c r="L20" s="23">
+        <v>0.69079999999999997</v>
+      </c>
+      <c r="M20" s="23">
+        <v>0.51400000000000001</v>
+      </c>
+      <c r="N20" s="23">
+        <v>0.13</v>
+      </c>
+      <c r="O20" s="23">
+        <v>0.35089999999999999</v>
+      </c>
+      <c r="P20" s="23">
+        <v>0.63719999999999999</v>
+      </c>
+      <c r="Q20" s="29"/>
+      <c r="R20" s="29"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A21" s="30">
+        <v>18</v>
+      </c>
+      <c r="B21" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="30">
+        <v>100</v>
+      </c>
+      <c r="E21" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="F21" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G21" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H21" s="24">
+        <v>0.42</v>
+      </c>
+      <c r="I21" s="24">
+        <v>0.52649999999999997</v>
+      </c>
+      <c r="J21" s="24">
+        <v>0.21</v>
+      </c>
+      <c r="K21" s="24">
+        <v>0.56779999999999997</v>
+      </c>
+      <c r="L21" s="24">
+        <v>0.70499999999999996</v>
+      </c>
+      <c r="M21" s="24">
+        <v>0.51149999999999995</v>
+      </c>
+      <c r="N21" s="24">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="O21" s="24">
+        <v>0.37030000000000002</v>
+      </c>
+      <c r="P21" s="24">
+        <v>0.65249999999999997</v>
+      </c>
+      <c r="Q21" s="30"/>
+      <c r="R21" s="30"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A22" s="31">
+        <v>19</v>
+      </c>
+      <c r="B22" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="31">
+        <v>100</v>
+      </c>
+      <c r="E22" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H22" s="25">
+        <v>0.42</v>
+      </c>
+      <c r="I22" s="25">
+        <v>0.56899999999999995</v>
+      </c>
+      <c r="J22" s="25">
+        <v>0.24</v>
+      </c>
+      <c r="K22" s="25">
+        <v>0.60970000000000002</v>
+      </c>
+      <c r="L22" s="25">
+        <v>0.71750000000000003</v>
+      </c>
+      <c r="M22" s="25">
+        <v>0.56320000000000003</v>
+      </c>
+      <c r="N22" s="25">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="O22" s="25">
+        <v>0.42320000000000002</v>
+      </c>
+      <c r="P22" s="25">
+        <v>0.65790000000000004</v>
+      </c>
+      <c r="Q22" s="31"/>
+      <c r="R22" s="31"/>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A23" s="30">
+        <v>20</v>
+      </c>
+      <c r="B23" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" s="30">
+        <v>100</v>
+      </c>
+      <c r="E23" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="F23" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H23" s="24">
+        <v>0.39</v>
+      </c>
+      <c r="I23" s="24">
+        <v>0.51259999999999994</v>
+      </c>
+      <c r="J23" s="24">
+        <v>0.17</v>
+      </c>
+      <c r="K23" s="24">
+        <v>0.5524</v>
+      </c>
+      <c r="L23" s="24">
+        <v>0.69330000000000003</v>
+      </c>
+      <c r="M23" s="24">
+        <v>0.49480000000000002</v>
+      </c>
+      <c r="N23" s="24">
+        <v>0.1</v>
+      </c>
+      <c r="O23" s="24">
+        <v>0.34329999999999999</v>
+      </c>
+      <c r="P23" s="24">
+        <v>0.61450000000000005</v>
+      </c>
+      <c r="Q23" s="30"/>
+      <c r="R23" s="30"/>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A25" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="22"/>
+      <c r="J25" s="22"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="22"/>
+      <c r="M25" s="22"/>
+      <c r="N25" s="22"/>
+      <c r="O25" s="22"/>
+      <c r="P25" s="22"/>
+      <c r="Q25" s="22"/>
+      <c r="R25" s="22"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A26" s="30">
+        <v>21</v>
+      </c>
+      <c r="B26" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="30">
+        <v>100</v>
+      </c>
+      <c r="E26" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="F26" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" s="24">
+        <v>0.43</v>
+      </c>
+      <c r="I26" s="24">
+        <v>0.55030000000000001</v>
+      </c>
+      <c r="J26" s="24">
+        <v>0.22</v>
+      </c>
+      <c r="K26" s="24">
+        <v>0.58140000000000003</v>
+      </c>
+      <c r="L26" s="24">
+        <v>0.69420000000000004</v>
+      </c>
+      <c r="M26" s="24">
+        <v>0.53400000000000003</v>
+      </c>
+      <c r="N26" s="24">
+        <v>0.11</v>
+      </c>
+      <c r="O26" s="24">
+        <v>0.39850000000000002</v>
+      </c>
+      <c r="P26" s="24">
+        <v>0.68079999999999996</v>
+      </c>
+      <c r="Q26" s="30"/>
+      <c r="R26" s="30"/>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A27" s="29">
+        <v>22</v>
+      </c>
+      <c r="B27" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="C27" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="29">
+        <v>100</v>
+      </c>
+      <c r="E27" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="F27" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" s="23">
+        <v>0.4</v>
+      </c>
+      <c r="I27" s="23">
+        <v>0.5474</v>
+      </c>
+      <c r="J27" s="23">
+        <v>0.21</v>
+      </c>
+      <c r="K27" s="23">
+        <v>0.58879999999999999</v>
+      </c>
+      <c r="L27" s="23">
+        <v>0.71499999999999997</v>
+      </c>
+      <c r="M27" s="23">
+        <v>0.53569999999999995</v>
+      </c>
+      <c r="N27" s="23">
+        <v>0.1</v>
+      </c>
+      <c r="O27" s="23">
+        <v>0.39069999999999999</v>
+      </c>
+      <c r="P27" s="23">
+        <v>0.67090000000000005</v>
+      </c>
+      <c r="Q27" s="29"/>
+      <c r="R27" s="29"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A28" s="30">
+        <v>23</v>
+      </c>
+      <c r="B28" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="30">
+        <v>100</v>
+      </c>
+      <c r="E28" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="F28" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H28" s="24">
+        <v>0.42</v>
+      </c>
+      <c r="I28" s="24">
+        <v>0.55940000000000001</v>
+      </c>
+      <c r="J28" s="24">
+        <v>0.25</v>
+      </c>
+      <c r="K28" s="24">
+        <v>0.59150000000000003</v>
+      </c>
+      <c r="L28" s="24">
+        <v>0.7</v>
+      </c>
+      <c r="M28" s="24">
+        <v>0.54069999999999996</v>
+      </c>
+      <c r="N28" s="24">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="O28" s="24">
+        <v>0.41739999999999999</v>
+      </c>
+      <c r="P28" s="24">
+        <v>0.69579999999999997</v>
+      </c>
+      <c r="Q28" s="30"/>
+      <c r="R28" s="30"/>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A29" s="31">
+        <v>24</v>
+      </c>
+      <c r="B29" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="C29" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="31">
+        <v>100</v>
+      </c>
+      <c r="E29" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="F29" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="G29" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H29" s="25">
+        <v>0.44</v>
+      </c>
+      <c r="I29" s="25">
+        <v>0.58989999999999998</v>
+      </c>
+      <c r="J29" s="25">
+        <v>0.27</v>
+      </c>
+      <c r="K29" s="25">
+        <v>0.61050000000000004</v>
+      </c>
+      <c r="L29" s="25">
+        <v>0.71</v>
+      </c>
+      <c r="M29" s="25">
+        <v>0.56320000000000003</v>
+      </c>
+      <c r="N29" s="25">
+        <v>0.15</v>
+      </c>
+      <c r="O29" s="25">
+        <v>0.44359999999999999</v>
+      </c>
+      <c r="P29" s="25">
+        <v>0.67830000000000001</v>
+      </c>
+      <c r="Q29" s="31"/>
+      <c r="R29" s="31"/>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A30" s="30">
+        <v>25</v>
+      </c>
+      <c r="B30" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D30" s="30">
+        <v>100</v>
+      </c>
+      <c r="E30" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="F30" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G30" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H30" s="24">
+        <v>0.41</v>
+      </c>
+      <c r="I30" s="24">
+        <v>0.56220000000000003</v>
+      </c>
+      <c r="J30" s="24">
+        <v>0.23</v>
+      </c>
+      <c r="K30" s="24">
+        <v>0.61009999999999998</v>
+      </c>
+      <c r="L30" s="24">
+        <v>0.73080000000000001</v>
+      </c>
+      <c r="M30" s="24">
+        <v>0.55479999999999996</v>
+      </c>
+      <c r="N30" s="24">
+        <v>0.12</v>
+      </c>
+      <c r="O30" s="24">
+        <v>0.41199999999999998</v>
+      </c>
+      <c r="P30" s="24">
+        <v>0.6542</v>
+      </c>
+      <c r="Q30" s="30"/>
+      <c r="R30" s="30"/>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A32" s="27" t="s">
+        <v>53</v>
+      </c>
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="22"/>
+      <c r="J32" s="22"/>
+      <c r="K32" s="22"/>
+      <c r="L32" s="22"/>
+      <c r="M32" s="22"/>
+      <c r="N32" s="22"/>
+      <c r="O32" s="22"/>
+      <c r="P32" s="22"/>
+      <c r="Q32" s="22"/>
+      <c r="R32" s="22"/>
+    </row>
+    <row r="33" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="31">
+        <v>26</v>
+      </c>
+      <c r="B33" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D33" s="31">
+        <v>100</v>
+      </c>
+      <c r="E33" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="F33" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="G33" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H33" s="25">
+        <v>0.52</v>
+      </c>
+      <c r="I33" s="25">
+        <v>0.64849999999999997</v>
+      </c>
+      <c r="J33" s="25">
+        <v>0.21</v>
+      </c>
+      <c r="K33" s="25">
+        <v>0.629</v>
+      </c>
+      <c r="L33" s="25">
+        <v>0.74419999999999997</v>
+      </c>
+      <c r="M33" s="25">
+        <v>0.57069999999999999</v>
+      </c>
+      <c r="N33" s="25">
+        <v>0.15</v>
+      </c>
+      <c r="O33" s="25">
+        <v>0.47189999999999999</v>
+      </c>
+      <c r="P33" s="25">
+        <v>0.74450000000000005</v>
+      </c>
+      <c r="Q33" s="31"/>
+      <c r="R33" s="31"/>
+    </row>
+    <row r="34" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="30">
+        <v>27</v>
+      </c>
+      <c r="B34" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C34" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D34" s="30">
+        <v>100</v>
+      </c>
+      <c r="E34" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G34" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H34" s="24">
+        <v>0.47</v>
+      </c>
+      <c r="I34" s="24">
+        <v>0.63339999999999996</v>
+      </c>
+      <c r="J34" s="24">
+        <v>0.27</v>
+      </c>
+      <c r="K34" s="24">
+        <v>0.63900000000000001</v>
+      </c>
+      <c r="L34" s="24">
+        <v>0.745</v>
+      </c>
+      <c r="M34" s="24">
+        <v>0.59230000000000005</v>
+      </c>
+      <c r="N34" s="24">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="O34" s="24">
+        <v>0.4647</v>
+      </c>
+      <c r="P34" s="24">
+        <v>0.7601</v>
+      </c>
+      <c r="Q34" s="30"/>
+      <c r="R34" s="30"/>
+    </row>
+    <row r="35" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="30">
+        <v>28</v>
+      </c>
+      <c r="B35" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C35" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" s="30">
+        <v>100</v>
+      </c>
+      <c r="E35" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="F35" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G35" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H35" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="I35" s="24">
+        <v>0.64810000000000001</v>
+      </c>
+      <c r="J35" s="24">
+        <v>0.27</v>
+      </c>
+      <c r="K35" s="24">
+        <v>0.63839999999999997</v>
+      </c>
+      <c r="L35" s="24">
+        <v>0.74580000000000002</v>
+      </c>
+      <c r="M35" s="24">
+        <v>0.58399999999999996</v>
+      </c>
+      <c r="N35" s="24">
+        <v>0.17</v>
+      </c>
+      <c r="O35" s="24">
+        <v>0.47449999999999998</v>
+      </c>
+      <c r="P35" s="24">
+        <v>0.67330000000000001</v>
+      </c>
+      <c r="Q35" s="30"/>
+      <c r="R35" s="30"/>
+    </row>
+    <row r="36" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="29">
+        <v>29</v>
+      </c>
+      <c r="B36" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C36" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="29">
+        <v>100</v>
+      </c>
+      <c r="E36" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="F36" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="G36" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="H36" s="23">
+        <v>0.45</v>
+      </c>
+      <c r="I36" s="23">
+        <v>0.61450000000000005</v>
+      </c>
+      <c r="J36" s="23">
+        <v>0.27</v>
+      </c>
+      <c r="K36" s="23">
+        <v>0.60840000000000005</v>
+      </c>
+      <c r="L36" s="23">
+        <v>0.71330000000000005</v>
+      </c>
+      <c r="M36" s="23">
+        <v>0.56030000000000002</v>
+      </c>
+      <c r="N36" s="23">
+        <v>0.15</v>
+      </c>
+      <c r="O36" s="23">
+        <v>0.43259999999999998</v>
+      </c>
+      <c r="P36" s="23">
+        <v>0.7167</v>
+      </c>
+      <c r="Q36" s="29"/>
+      <c r="R36" s="29"/>
+    </row>
+    <row r="37" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A37" s="30">
+        <v>30</v>
+      </c>
+      <c r="B37" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C37" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="30">
+        <v>100</v>
+      </c>
+      <c r="E37" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="F37" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G37" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H37" s="24">
+        <v>0.48</v>
+      </c>
+      <c r="I37" s="24">
+        <v>0.63029999999999997</v>
+      </c>
+      <c r="J37" s="24">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="K37" s="24">
+        <v>0.62870000000000004</v>
+      </c>
+      <c r="L37" s="24">
+        <v>0.74170000000000003</v>
+      </c>
+      <c r="M37" s="24">
+        <v>0.57650000000000001</v>
+      </c>
+      <c r="N37" s="24">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="O37" s="24">
+        <v>0.46479999999999999</v>
+      </c>
+      <c r="P37" s="24">
+        <v>0.67600000000000005</v>
+      </c>
+      <c r="Q37" s="30"/>
+      <c r="R37" s="30"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A4:R4"/>
+    <mergeCell ref="A11:R11"/>
+    <mergeCell ref="A18:R18"/>
+    <mergeCell ref="A25:R25"/>
+    <mergeCell ref="A32:R32"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>